<commit_message>
Fixture: Rules sheet, Include Expressions and Variables columns, schedule unchanged
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixture/sample-value-stream.xlsx
+++ b/fixture/sample-value-stream.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task List" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toggles" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Matrix" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary by Phase" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Task List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Edges" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Toggles" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Rules" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Profiles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Scenario Matrix" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Assumptions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Summary by Phase" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y147"/>
+  <dimension ref="A1:AE147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -459,6 +460,12 @@
     <col width="10" customWidth="1" min="23" max="23"/>
     <col width="11" customWidth="1" min="24" max="24"/>
     <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="24" customWidth="1" min="27" max="27"/>
+    <col width="34" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="11" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -587,6 +594,36 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Rule ID</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Include Expression</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Trigger Explanation</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Default Included</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Can Override</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Rule Priority</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -680,6 +717,12 @@
         </is>
       </c>
       <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -773,6 +816,12 @@
       </c>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -866,6 +915,12 @@
       </c>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -963,6 +1018,12 @@
         </is>
       </c>
       <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1060,6 +1121,12 @@
         </is>
       </c>
       <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1157,6 +1224,12 @@
         </is>
       </c>
       <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1254,6 +1327,12 @@
         </is>
       </c>
       <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1351,6 +1430,12 @@
         </is>
       </c>
       <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1448,6 +1533,12 @@
         </is>
       </c>
       <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1545,6 +1636,12 @@
         </is>
       </c>
       <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1642,6 +1739,12 @@
         </is>
       </c>
       <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1739,6 +1842,12 @@
         </is>
       </c>
       <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1836,6 +1945,20 @@
         </is>
       </c>
       <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>genAI = true</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>AI governance applies to generative AI workloads</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1933,6 +2056,12 @@
         </is>
       </c>
       <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2030,6 +2159,12 @@
         </is>
       </c>
       <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2127,6 +2262,12 @@
         </is>
       </c>
       <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2224,6 +2365,12 @@
         </is>
       </c>
       <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2321,6 +2468,12 @@
         </is>
       </c>
       <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2414,6 +2567,12 @@
       </c>
       <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2511,6 +2670,12 @@
         </is>
       </c>
       <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2604,6 +2769,12 @@
       </c>
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2701,6 +2872,12 @@
         </is>
       </c>
       <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2798,6 +2975,12 @@
         </is>
       </c>
       <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2895,6 +3078,12 @@
         </is>
       </c>
       <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2992,6 +3181,12 @@
         </is>
       </c>
       <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3089,6 +3284,12 @@
         </is>
       </c>
       <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3186,6 +3387,12 @@
         </is>
       </c>
       <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3283,6 +3490,12 @@
         </is>
       </c>
       <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
+      <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3376,6 +3589,12 @@
       </c>
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
+      <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3473,6 +3692,12 @@
         </is>
       </c>
       <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr"/>
+      <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -3566,6 +3791,12 @@
       </c>
       <c r="X32" t="inlineStr"/>
       <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
+      <c r="AD32" t="inlineStr"/>
+      <c r="AE32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3663,6 +3894,12 @@
         </is>
       </c>
       <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr"/>
+      <c r="AD33" t="inlineStr"/>
+      <c r="AE33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -3760,6 +3997,12 @@
         </is>
       </c>
       <c r="Y34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr"/>
+      <c r="AD34" t="inlineStr"/>
+      <c r="AE34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -3857,6 +4100,12 @@
         </is>
       </c>
       <c r="Y35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr"/>
+      <c r="AD35" t="inlineStr"/>
+      <c r="AE35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3954,6 +4203,12 @@
         </is>
       </c>
       <c r="Y36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr"/>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr"/>
+      <c r="AD36" t="inlineStr"/>
+      <c r="AE36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -4051,6 +4306,12 @@
         </is>
       </c>
       <c r="Y37" t="inlineStr"/>
+      <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="inlineStr"/>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr"/>
+      <c r="AD37" t="inlineStr"/>
+      <c r="AE37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -4148,6 +4409,12 @@
         </is>
       </c>
       <c r="Y38" t="inlineStr"/>
+      <c r="Z38" t="inlineStr"/>
+      <c r="AA38" t="inlineStr"/>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr"/>
+      <c r="AD38" t="inlineStr"/>
+      <c r="AE38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -4241,6 +4508,12 @@
       </c>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="inlineStr"/>
+      <c r="Z39" t="inlineStr"/>
+      <c r="AA39" t="inlineStr"/>
+      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr"/>
+      <c r="AD39" t="inlineStr"/>
+      <c r="AE39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -4338,6 +4611,12 @@
         </is>
       </c>
       <c r="Y40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr"/>
+      <c r="AA40" t="inlineStr"/>
+      <c r="AB40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr"/>
+      <c r="AD40" t="inlineStr"/>
+      <c r="AE40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -4435,6 +4714,12 @@
         </is>
       </c>
       <c r="Y41" t="inlineStr"/>
+      <c r="Z41" t="inlineStr"/>
+      <c r="AA41" t="inlineStr"/>
+      <c r="AB41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr"/>
+      <c r="AD41" t="inlineStr"/>
+      <c r="AE41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -4528,6 +4813,12 @@
       </c>
       <c r="X42" t="inlineStr"/>
       <c r="Y42" t="inlineStr"/>
+      <c r="Z42" t="inlineStr"/>
+      <c r="AA42" t="inlineStr"/>
+      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr"/>
+      <c r="AD42" t="inlineStr"/>
+      <c r="AE42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -4621,6 +4912,12 @@
       </c>
       <c r="X43" t="inlineStr"/>
       <c r="Y43" t="inlineStr"/>
+      <c r="Z43" t="inlineStr"/>
+      <c r="AA43" t="inlineStr"/>
+      <c r="AB43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr"/>
+      <c r="AD43" t="inlineStr"/>
+      <c r="AE43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -4718,6 +5015,12 @@
         </is>
       </c>
       <c r="Y44" t="inlineStr"/>
+      <c r="Z44" t="inlineStr"/>
+      <c r="AA44" t="inlineStr"/>
+      <c r="AB44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr"/>
+      <c r="AD44" t="inlineStr"/>
+      <c r="AE44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -4815,6 +5118,12 @@
         </is>
       </c>
       <c r="Y45" t="inlineStr"/>
+      <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="inlineStr"/>
+      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr"/>
+      <c r="AD45" t="inlineStr"/>
+      <c r="AE45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -4912,6 +5221,12 @@
         </is>
       </c>
       <c r="Y46" t="inlineStr"/>
+      <c r="Z46" t="inlineStr"/>
+      <c r="AA46" t="inlineStr"/>
+      <c r="AB46" t="inlineStr"/>
+      <c r="AC46" t="inlineStr"/>
+      <c r="AD46" t="inlineStr"/>
+      <c r="AE46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -5009,6 +5324,12 @@
         </is>
       </c>
       <c r="Y47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr"/>
+      <c r="AA47" t="inlineStr"/>
+      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr"/>
+      <c r="AD47" t="inlineStr"/>
+      <c r="AE47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -5106,6 +5427,12 @@
         </is>
       </c>
       <c r="Y48" t="inlineStr"/>
+      <c r="Z48" t="inlineStr"/>
+      <c r="AA48" t="inlineStr"/>
+      <c r="AB48" t="inlineStr"/>
+      <c r="AC48" t="inlineStr"/>
+      <c r="AD48" t="inlineStr"/>
+      <c r="AE48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -5199,6 +5526,12 @@
       </c>
       <c r="X49" t="inlineStr"/>
       <c r="Y49" t="inlineStr"/>
+      <c r="Z49" t="inlineStr"/>
+      <c r="AA49" t="inlineStr"/>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr"/>
+      <c r="AD49" t="inlineStr"/>
+      <c r="AE49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -5296,6 +5629,12 @@
         </is>
       </c>
       <c r="Y50" t="inlineStr"/>
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr"/>
+      <c r="AD50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -5389,6 +5728,12 @@
       </c>
       <c r="X51" t="inlineStr"/>
       <c r="Y51" t="inlineStr"/>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr"/>
+      <c r="AD51" t="inlineStr"/>
+      <c r="AE51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -5482,6 +5827,12 @@
       </c>
       <c r="X52" t="inlineStr"/>
       <c r="Y52" t="inlineStr"/>
+      <c r="Z52" t="inlineStr"/>
+      <c r="AA52" t="inlineStr"/>
+      <c r="AB52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr"/>
+      <c r="AD52" t="inlineStr"/>
+      <c r="AE52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -5575,6 +5926,20 @@
       </c>
       <c r="X53" t="inlineStr"/>
       <c r="Y53" t="inlineStr"/>
+      <c r="Z53" t="inlineStr"/>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>genAI = true</t>
+        </is>
+      </c>
+      <c r="AB53" t="inlineStr">
+        <is>
+          <t>AI governance applies to generative AI workloads</t>
+        </is>
+      </c>
+      <c r="AC53" t="inlineStr"/>
+      <c r="AD53" t="inlineStr"/>
+      <c r="AE53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -5668,6 +6033,12 @@
       </c>
       <c r="X54" t="inlineStr"/>
       <c r="Y54" t="inlineStr"/>
+      <c r="Z54" t="inlineStr"/>
+      <c r="AA54" t="inlineStr"/>
+      <c r="AB54" t="inlineStr"/>
+      <c r="AC54" t="inlineStr"/>
+      <c r="AD54" t="inlineStr"/>
+      <c r="AE54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -5761,6 +6132,12 @@
       </c>
       <c r="X55" t="inlineStr"/>
       <c r="Y55" t="inlineStr"/>
+      <c r="Z55" t="inlineStr"/>
+      <c r="AA55" t="inlineStr"/>
+      <c r="AB55" t="inlineStr"/>
+      <c r="AC55" t="inlineStr"/>
+      <c r="AD55" t="inlineStr"/>
+      <c r="AE55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -5858,6 +6235,12 @@
         </is>
       </c>
       <c r="Y56" t="inlineStr"/>
+      <c r="Z56" t="inlineStr"/>
+      <c r="AA56" t="inlineStr"/>
+      <c r="AB56" t="inlineStr"/>
+      <c r="AC56" t="inlineStr"/>
+      <c r="AD56" t="inlineStr"/>
+      <c r="AE56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -5951,6 +6334,12 @@
       </c>
       <c r="X57" t="inlineStr"/>
       <c r="Y57" t="inlineStr"/>
+      <c r="Z57" t="inlineStr"/>
+      <c r="AA57" t="inlineStr"/>
+      <c r="AB57" t="inlineStr"/>
+      <c r="AC57" t="inlineStr"/>
+      <c r="AD57" t="inlineStr"/>
+      <c r="AE57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -6048,6 +6437,12 @@
         </is>
       </c>
       <c r="Y58" t="inlineStr"/>
+      <c r="Z58" t="inlineStr"/>
+      <c r="AA58" t="inlineStr"/>
+      <c r="AB58" t="inlineStr"/>
+      <c r="AC58" t="inlineStr"/>
+      <c r="AD58" t="inlineStr"/>
+      <c r="AE58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -6141,6 +6536,12 @@
       </c>
       <c r="X59" t="inlineStr"/>
       <c r="Y59" t="inlineStr"/>
+      <c r="Z59" t="inlineStr"/>
+      <c r="AA59" t="inlineStr"/>
+      <c r="AB59" t="inlineStr"/>
+      <c r="AC59" t="inlineStr"/>
+      <c r="AD59" t="inlineStr"/>
+      <c r="AE59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -6238,6 +6639,12 @@
         </is>
       </c>
       <c r="Y60" t="inlineStr"/>
+      <c r="Z60" t="inlineStr"/>
+      <c r="AA60" t="inlineStr"/>
+      <c r="AB60" t="inlineStr"/>
+      <c r="AC60" t="inlineStr"/>
+      <c r="AD60" t="inlineStr"/>
+      <c r="AE60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -6335,6 +6742,12 @@
         </is>
       </c>
       <c r="Y61" t="inlineStr"/>
+      <c r="Z61" t="inlineStr"/>
+      <c r="AA61" t="inlineStr"/>
+      <c r="AB61" t="inlineStr"/>
+      <c r="AC61" t="inlineStr"/>
+      <c r="AD61" t="inlineStr"/>
+      <c r="AE61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -6432,6 +6845,12 @@
         </is>
       </c>
       <c r="Y62" t="inlineStr"/>
+      <c r="Z62" t="inlineStr"/>
+      <c r="AA62" t="inlineStr"/>
+      <c r="AB62" t="inlineStr"/>
+      <c r="AC62" t="inlineStr"/>
+      <c r="AD62" t="inlineStr"/>
+      <c r="AE62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -6529,6 +6948,12 @@
         </is>
       </c>
       <c r="Y63" t="inlineStr"/>
+      <c r="Z63" t="inlineStr"/>
+      <c r="AA63" t="inlineStr"/>
+      <c r="AB63" t="inlineStr"/>
+      <c r="AC63" t="inlineStr"/>
+      <c r="AD63" t="inlineStr"/>
+      <c r="AE63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -6626,6 +7051,12 @@
         </is>
       </c>
       <c r="Y64" t="inlineStr"/>
+      <c r="Z64" t="inlineStr"/>
+      <c r="AA64" t="inlineStr"/>
+      <c r="AB64" t="inlineStr"/>
+      <c r="AC64" t="inlineStr"/>
+      <c r="AD64" t="inlineStr"/>
+      <c r="AE64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -6723,6 +7154,12 @@
         </is>
       </c>
       <c r="Y65" t="inlineStr"/>
+      <c r="Z65" t="inlineStr"/>
+      <c r="AA65" t="inlineStr"/>
+      <c r="AB65" t="inlineStr"/>
+      <c r="AC65" t="inlineStr"/>
+      <c r="AD65" t="inlineStr"/>
+      <c r="AE65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -6820,6 +7257,20 @@
         </is>
       </c>
       <c r="Y66" t="inlineStr"/>
+      <c r="Z66" t="inlineStr"/>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>genAI = true</t>
+        </is>
+      </c>
+      <c r="AB66" t="inlineStr">
+        <is>
+          <t>AI governance applies to generative AI workloads</t>
+        </is>
+      </c>
+      <c r="AC66" t="inlineStr"/>
+      <c r="AD66" t="inlineStr"/>
+      <c r="AE66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -6917,6 +7368,12 @@
         </is>
       </c>
       <c r="Y67" t="inlineStr"/>
+      <c r="Z67" t="inlineStr"/>
+      <c r="AA67" t="inlineStr"/>
+      <c r="AB67" t="inlineStr"/>
+      <c r="AC67" t="inlineStr"/>
+      <c r="AD67" t="inlineStr"/>
+      <c r="AE67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -7014,6 +7471,12 @@
         </is>
       </c>
       <c r="Y68" t="inlineStr"/>
+      <c r="Z68" t="inlineStr"/>
+      <c r="AA68" t="inlineStr"/>
+      <c r="AB68" t="inlineStr"/>
+      <c r="AC68" t="inlineStr"/>
+      <c r="AD68" t="inlineStr"/>
+      <c r="AE68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -7107,6 +7570,12 @@
       </c>
       <c r="X69" t="inlineStr"/>
       <c r="Y69" t="inlineStr"/>
+      <c r="Z69" t="inlineStr"/>
+      <c r="AA69" t="inlineStr"/>
+      <c r="AB69" t="inlineStr"/>
+      <c r="AC69" t="inlineStr"/>
+      <c r="AD69" t="inlineStr"/>
+      <c r="AE69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -7204,6 +7673,12 @@
         </is>
       </c>
       <c r="Y70" t="inlineStr"/>
+      <c r="Z70" t="inlineStr"/>
+      <c r="AA70" t="inlineStr"/>
+      <c r="AB70" t="inlineStr"/>
+      <c r="AC70" t="inlineStr"/>
+      <c r="AD70" t="inlineStr"/>
+      <c r="AE70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -7301,6 +7776,12 @@
         </is>
       </c>
       <c r="Y71" t="inlineStr"/>
+      <c r="Z71" t="inlineStr"/>
+      <c r="AA71" t="inlineStr"/>
+      <c r="AB71" t="inlineStr"/>
+      <c r="AC71" t="inlineStr"/>
+      <c r="AD71" t="inlineStr"/>
+      <c r="AE71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -7398,6 +7879,16 @@
         </is>
       </c>
       <c r="Y72" t="inlineStr"/>
+      <c r="Z72" t="inlineStr"/>
+      <c r="AA72" t="inlineStr"/>
+      <c r="AB72" t="inlineStr"/>
+      <c r="AC72" t="inlineStr"/>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t>Governed</t>
+        </is>
+      </c>
+      <c r="AE72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -7495,6 +7986,16 @@
         </is>
       </c>
       <c r="Y73" t="inlineStr"/>
+      <c r="Z73" t="inlineStr"/>
+      <c r="AA73" t="inlineStr"/>
+      <c r="AB73" t="inlineStr"/>
+      <c r="AC73" t="inlineStr"/>
+      <c r="AD73" t="inlineStr">
+        <is>
+          <t>Governed</t>
+        </is>
+      </c>
+      <c r="AE73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -7592,6 +8093,16 @@
         </is>
       </c>
       <c r="Y74" t="inlineStr"/>
+      <c r="Z74" t="inlineStr"/>
+      <c r="AA74" t="inlineStr"/>
+      <c r="AB74" t="inlineStr"/>
+      <c r="AC74" t="inlineStr"/>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t>Governed</t>
+        </is>
+      </c>
+      <c r="AE74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -7689,6 +8200,12 @@
         </is>
       </c>
       <c r="Y75" t="inlineStr"/>
+      <c r="Z75" t="inlineStr"/>
+      <c r="AA75" t="inlineStr"/>
+      <c r="AB75" t="inlineStr"/>
+      <c r="AC75" t="inlineStr"/>
+      <c r="AD75" t="inlineStr"/>
+      <c r="AE75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -7786,6 +8303,12 @@
         </is>
       </c>
       <c r="Y76" t="inlineStr"/>
+      <c r="Z76" t="inlineStr"/>
+      <c r="AA76" t="inlineStr"/>
+      <c r="AB76" t="inlineStr"/>
+      <c r="AC76" t="inlineStr"/>
+      <c r="AD76" t="inlineStr"/>
+      <c r="AE76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -7879,6 +8402,12 @@
       </c>
       <c r="X77" t="inlineStr"/>
       <c r="Y77" t="inlineStr"/>
+      <c r="Z77" t="inlineStr"/>
+      <c r="AA77" t="inlineStr"/>
+      <c r="AB77" t="inlineStr"/>
+      <c r="AC77" t="inlineStr"/>
+      <c r="AD77" t="inlineStr"/>
+      <c r="AE77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -7972,6 +8501,12 @@
       </c>
       <c r="X78" t="inlineStr"/>
       <c r="Y78" t="inlineStr"/>
+      <c r="Z78" t="inlineStr"/>
+      <c r="AA78" t="inlineStr"/>
+      <c r="AB78" t="inlineStr"/>
+      <c r="AC78" t="inlineStr"/>
+      <c r="AD78" t="inlineStr"/>
+      <c r="AE78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -8065,6 +8600,12 @@
       </c>
       <c r="X79" t="inlineStr"/>
       <c r="Y79" t="inlineStr"/>
+      <c r="Z79" t="inlineStr"/>
+      <c r="AA79" t="inlineStr"/>
+      <c r="AB79" t="inlineStr"/>
+      <c r="AC79" t="inlineStr"/>
+      <c r="AD79" t="inlineStr"/>
+      <c r="AE79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -8162,6 +8703,12 @@
         </is>
       </c>
       <c r="Y80" t="inlineStr"/>
+      <c r="Z80" t="inlineStr"/>
+      <c r="AA80" t="inlineStr"/>
+      <c r="AB80" t="inlineStr"/>
+      <c r="AC80" t="inlineStr"/>
+      <c r="AD80" t="inlineStr"/>
+      <c r="AE80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -8259,6 +8806,12 @@
         </is>
       </c>
       <c r="Y81" t="inlineStr"/>
+      <c r="Z81" t="inlineStr"/>
+      <c r="AA81" t="inlineStr"/>
+      <c r="AB81" t="inlineStr"/>
+      <c r="AC81" t="inlineStr"/>
+      <c r="AD81" t="inlineStr"/>
+      <c r="AE81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -8352,6 +8905,12 @@
       </c>
       <c r="X82" t="inlineStr"/>
       <c r="Y82" t="inlineStr"/>
+      <c r="Z82" t="inlineStr"/>
+      <c r="AA82" t="inlineStr"/>
+      <c r="AB82" t="inlineStr"/>
+      <c r="AC82" t="inlineStr"/>
+      <c r="AD82" t="inlineStr"/>
+      <c r="AE82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -8449,6 +9008,12 @@
         </is>
       </c>
       <c r="Y83" t="inlineStr"/>
+      <c r="Z83" t="inlineStr"/>
+      <c r="AA83" t="inlineStr"/>
+      <c r="AB83" t="inlineStr"/>
+      <c r="AC83" t="inlineStr"/>
+      <c r="AD83" t="inlineStr"/>
+      <c r="AE83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -8546,6 +9111,12 @@
         </is>
       </c>
       <c r="Y84" t="inlineStr"/>
+      <c r="Z84" t="inlineStr"/>
+      <c r="AA84" t="inlineStr"/>
+      <c r="AB84" t="inlineStr"/>
+      <c r="AC84" t="inlineStr"/>
+      <c r="AD84" t="inlineStr"/>
+      <c r="AE84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -8643,6 +9214,12 @@
         </is>
       </c>
       <c r="Y85" t="inlineStr"/>
+      <c r="Z85" t="inlineStr"/>
+      <c r="AA85" t="inlineStr"/>
+      <c r="AB85" t="inlineStr"/>
+      <c r="AC85" t="inlineStr"/>
+      <c r="AD85" t="inlineStr"/>
+      <c r="AE85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -8740,6 +9317,12 @@
         </is>
       </c>
       <c r="Y86" t="inlineStr"/>
+      <c r="Z86" t="inlineStr"/>
+      <c r="AA86" t="inlineStr"/>
+      <c r="AB86" t="inlineStr"/>
+      <c r="AC86" t="inlineStr"/>
+      <c r="AD86" t="inlineStr"/>
+      <c r="AE86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -8833,6 +9416,12 @@
       </c>
       <c r="X87" t="inlineStr"/>
       <c r="Y87" t="inlineStr"/>
+      <c r="Z87" t="inlineStr"/>
+      <c r="AA87" t="inlineStr"/>
+      <c r="AB87" t="inlineStr"/>
+      <c r="AC87" t="inlineStr"/>
+      <c r="AD87" t="inlineStr"/>
+      <c r="AE87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -8926,6 +9515,12 @@
       </c>
       <c r="X88" t="inlineStr"/>
       <c r="Y88" t="inlineStr"/>
+      <c r="Z88" t="inlineStr"/>
+      <c r="AA88" t="inlineStr"/>
+      <c r="AB88" t="inlineStr"/>
+      <c r="AC88" t="inlineStr"/>
+      <c r="AD88" t="inlineStr"/>
+      <c r="AE88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -9019,6 +9614,12 @@
       </c>
       <c r="X89" t="inlineStr"/>
       <c r="Y89" t="inlineStr"/>
+      <c r="Z89" t="inlineStr"/>
+      <c r="AA89" t="inlineStr"/>
+      <c r="AB89" t="inlineStr"/>
+      <c r="AC89" t="inlineStr"/>
+      <c r="AD89" t="inlineStr"/>
+      <c r="AE89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -9116,6 +9717,12 @@
         </is>
       </c>
       <c r="Y90" t="inlineStr"/>
+      <c r="Z90" t="inlineStr"/>
+      <c r="AA90" t="inlineStr"/>
+      <c r="AB90" t="inlineStr"/>
+      <c r="AC90" t="inlineStr"/>
+      <c r="AD90" t="inlineStr"/>
+      <c r="AE90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -9213,6 +9820,12 @@
         </is>
       </c>
       <c r="Y91" t="inlineStr"/>
+      <c r="Z91" t="inlineStr"/>
+      <c r="AA91" t="inlineStr"/>
+      <c r="AB91" t="inlineStr"/>
+      <c r="AC91" t="inlineStr"/>
+      <c r="AD91" t="inlineStr"/>
+      <c r="AE91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -9310,6 +9923,12 @@
         </is>
       </c>
       <c r="Y92" t="inlineStr"/>
+      <c r="Z92" t="inlineStr"/>
+      <c r="AA92" t="inlineStr"/>
+      <c r="AB92" t="inlineStr"/>
+      <c r="AC92" t="inlineStr"/>
+      <c r="AD92" t="inlineStr"/>
+      <c r="AE92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -9403,6 +10022,12 @@
       </c>
       <c r="X93" t="inlineStr"/>
       <c r="Y93" t="inlineStr"/>
+      <c r="Z93" t="inlineStr"/>
+      <c r="AA93" t="inlineStr"/>
+      <c r="AB93" t="inlineStr"/>
+      <c r="AC93" t="inlineStr"/>
+      <c r="AD93" t="inlineStr"/>
+      <c r="AE93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -9496,6 +10121,12 @@
       </c>
       <c r="X94" t="inlineStr"/>
       <c r="Y94" t="inlineStr"/>
+      <c r="Z94" t="inlineStr"/>
+      <c r="AA94" t="inlineStr"/>
+      <c r="AB94" t="inlineStr"/>
+      <c r="AC94" t="inlineStr"/>
+      <c r="AD94" t="inlineStr"/>
+      <c r="AE94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -9589,6 +10220,12 @@
       </c>
       <c r="X95" t="inlineStr"/>
       <c r="Y95" t="inlineStr"/>
+      <c r="Z95" t="inlineStr"/>
+      <c r="AA95" t="inlineStr"/>
+      <c r="AB95" t="inlineStr"/>
+      <c r="AC95" t="inlineStr"/>
+      <c r="AD95" t="inlineStr"/>
+      <c r="AE95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -9682,6 +10319,12 @@
       </c>
       <c r="X96" t="inlineStr"/>
       <c r="Y96" t="inlineStr"/>
+      <c r="Z96" t="inlineStr"/>
+      <c r="AA96" t="inlineStr"/>
+      <c r="AB96" t="inlineStr"/>
+      <c r="AC96" t="inlineStr"/>
+      <c r="AD96" t="inlineStr"/>
+      <c r="AE96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -9779,6 +10422,12 @@
         </is>
       </c>
       <c r="Y97" t="inlineStr"/>
+      <c r="Z97" t="inlineStr"/>
+      <c r="AA97" t="inlineStr"/>
+      <c r="AB97" t="inlineStr"/>
+      <c r="AC97" t="inlineStr"/>
+      <c r="AD97" t="inlineStr"/>
+      <c r="AE97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -9876,6 +10525,12 @@
         </is>
       </c>
       <c r="Y98" t="inlineStr"/>
+      <c r="Z98" t="inlineStr"/>
+      <c r="AA98" t="inlineStr"/>
+      <c r="AB98" t="inlineStr"/>
+      <c r="AC98" t="inlineStr"/>
+      <c r="AD98" t="inlineStr"/>
+      <c r="AE98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -9973,6 +10628,12 @@
         </is>
       </c>
       <c r="Y99" t="inlineStr"/>
+      <c r="Z99" t="inlineStr"/>
+      <c r="AA99" t="inlineStr"/>
+      <c r="AB99" t="inlineStr"/>
+      <c r="AC99" t="inlineStr"/>
+      <c r="AD99" t="inlineStr"/>
+      <c r="AE99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -10070,6 +10731,12 @@
         </is>
       </c>
       <c r="Y100" t="inlineStr"/>
+      <c r="Z100" t="inlineStr"/>
+      <c r="AA100" t="inlineStr"/>
+      <c r="AB100" t="inlineStr"/>
+      <c r="AC100" t="inlineStr"/>
+      <c r="AD100" t="inlineStr"/>
+      <c r="AE100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -10167,6 +10834,12 @@
         </is>
       </c>
       <c r="Y101" t="inlineStr"/>
+      <c r="Z101" t="inlineStr"/>
+      <c r="AA101" t="inlineStr"/>
+      <c r="AB101" t="inlineStr"/>
+      <c r="AC101" t="inlineStr"/>
+      <c r="AD101" t="inlineStr"/>
+      <c r="AE101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -10264,6 +10937,12 @@
         </is>
       </c>
       <c r="Y102" t="inlineStr"/>
+      <c r="Z102" t="inlineStr"/>
+      <c r="AA102" t="inlineStr"/>
+      <c r="AB102" t="inlineStr"/>
+      <c r="AC102" t="inlineStr"/>
+      <c r="AD102" t="inlineStr"/>
+      <c r="AE102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -10357,6 +11036,12 @@
       </c>
       <c r="X103" t="inlineStr"/>
       <c r="Y103" t="inlineStr"/>
+      <c r="Z103" t="inlineStr"/>
+      <c r="AA103" t="inlineStr"/>
+      <c r="AB103" t="inlineStr"/>
+      <c r="AC103" t="inlineStr"/>
+      <c r="AD103" t="inlineStr"/>
+      <c r="AE103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -10454,6 +11139,12 @@
         </is>
       </c>
       <c r="Y104" t="inlineStr"/>
+      <c r="Z104" t="inlineStr"/>
+      <c r="AA104" t="inlineStr"/>
+      <c r="AB104" t="inlineStr"/>
+      <c r="AC104" t="inlineStr"/>
+      <c r="AD104" t="inlineStr"/>
+      <c r="AE104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -10551,6 +11242,12 @@
         </is>
       </c>
       <c r="Y105" t="inlineStr"/>
+      <c r="Z105" t="inlineStr"/>
+      <c r="AA105" t="inlineStr"/>
+      <c r="AB105" t="inlineStr"/>
+      <c r="AC105" t="inlineStr"/>
+      <c r="AD105" t="inlineStr"/>
+      <c r="AE105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -10644,6 +11341,12 @@
       </c>
       <c r="X106" t="inlineStr"/>
       <c r="Y106" t="inlineStr"/>
+      <c r="Z106" t="inlineStr"/>
+      <c r="AA106" t="inlineStr"/>
+      <c r="AB106" t="inlineStr"/>
+      <c r="AC106" t="inlineStr"/>
+      <c r="AD106" t="inlineStr"/>
+      <c r="AE106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -10741,6 +11444,12 @@
         </is>
       </c>
       <c r="Y107" t="inlineStr"/>
+      <c r="Z107" t="inlineStr"/>
+      <c r="AA107" t="inlineStr"/>
+      <c r="AB107" t="inlineStr"/>
+      <c r="AC107" t="inlineStr"/>
+      <c r="AD107" t="inlineStr"/>
+      <c r="AE107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -10838,6 +11547,12 @@
         </is>
       </c>
       <c r="Y108" t="inlineStr"/>
+      <c r="Z108" t="inlineStr"/>
+      <c r="AA108" t="inlineStr"/>
+      <c r="AB108" t="inlineStr"/>
+      <c r="AC108" t="inlineStr"/>
+      <c r="AD108" t="inlineStr"/>
+      <c r="AE108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -10931,6 +11646,12 @@
       </c>
       <c r="X109" t="inlineStr"/>
       <c r="Y109" t="inlineStr"/>
+      <c r="Z109" t="inlineStr"/>
+      <c r="AA109" t="inlineStr"/>
+      <c r="AB109" t="inlineStr"/>
+      <c r="AC109" t="inlineStr"/>
+      <c r="AD109" t="inlineStr"/>
+      <c r="AE109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -11028,6 +11749,12 @@
         </is>
       </c>
       <c r="Y110" t="inlineStr"/>
+      <c r="Z110" t="inlineStr"/>
+      <c r="AA110" t="inlineStr"/>
+      <c r="AB110" t="inlineStr"/>
+      <c r="AC110" t="inlineStr"/>
+      <c r="AD110" t="inlineStr"/>
+      <c r="AE110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -11125,6 +11852,12 @@
         </is>
       </c>
       <c r="Y111" t="inlineStr"/>
+      <c r="Z111" t="inlineStr"/>
+      <c r="AA111" t="inlineStr"/>
+      <c r="AB111" t="inlineStr"/>
+      <c r="AC111" t="inlineStr"/>
+      <c r="AD111" t="inlineStr"/>
+      <c r="AE111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -11218,6 +11951,12 @@
       </c>
       <c r="X112" t="inlineStr"/>
       <c r="Y112" t="inlineStr"/>
+      <c r="Z112" t="inlineStr"/>
+      <c r="AA112" t="inlineStr"/>
+      <c r="AB112" t="inlineStr"/>
+      <c r="AC112" t="inlineStr"/>
+      <c r="AD112" t="inlineStr"/>
+      <c r="AE112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -11315,6 +12054,12 @@
         </is>
       </c>
       <c r="Y113" t="inlineStr"/>
+      <c r="Z113" t="inlineStr"/>
+      <c r="AA113" t="inlineStr"/>
+      <c r="AB113" t="inlineStr"/>
+      <c r="AC113" t="inlineStr"/>
+      <c r="AD113" t="inlineStr"/>
+      <c r="AE113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -11412,6 +12157,12 @@
         </is>
       </c>
       <c r="Y114" t="inlineStr"/>
+      <c r="Z114" t="inlineStr"/>
+      <c r="AA114" t="inlineStr"/>
+      <c r="AB114" t="inlineStr"/>
+      <c r="AC114" t="inlineStr"/>
+      <c r="AD114" t="inlineStr"/>
+      <c r="AE114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -11509,6 +12260,12 @@
         </is>
       </c>
       <c r="Y115" t="inlineStr"/>
+      <c r="Z115" t="inlineStr"/>
+      <c r="AA115" t="inlineStr"/>
+      <c r="AB115" t="inlineStr"/>
+      <c r="AC115" t="inlineStr"/>
+      <c r="AD115" t="inlineStr"/>
+      <c r="AE115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -11602,6 +12359,12 @@
       </c>
       <c r="X116" t="inlineStr"/>
       <c r="Y116" t="inlineStr"/>
+      <c r="Z116" t="inlineStr"/>
+      <c r="AA116" t="inlineStr"/>
+      <c r="AB116" t="inlineStr"/>
+      <c r="AC116" t="inlineStr"/>
+      <c r="AD116" t="inlineStr"/>
+      <c r="AE116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -11695,6 +12458,12 @@
       </c>
       <c r="X117" t="inlineStr"/>
       <c r="Y117" t="inlineStr"/>
+      <c r="Z117" t="inlineStr"/>
+      <c r="AA117" t="inlineStr"/>
+      <c r="AB117" t="inlineStr"/>
+      <c r="AC117" t="inlineStr"/>
+      <c r="AD117" t="inlineStr"/>
+      <c r="AE117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -11792,6 +12561,20 @@
         </is>
       </c>
       <c r="Y118" t="inlineStr"/>
+      <c r="Z118" t="inlineStr"/>
+      <c r="AA118" t="inlineStr">
+        <is>
+          <t>genAI = true</t>
+        </is>
+      </c>
+      <c r="AB118" t="inlineStr">
+        <is>
+          <t>AI governance applies to generative AI workloads</t>
+        </is>
+      </c>
+      <c r="AC118" t="inlineStr"/>
+      <c r="AD118" t="inlineStr"/>
+      <c r="AE118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -11889,6 +12672,12 @@
         </is>
       </c>
       <c r="Y119" t="inlineStr"/>
+      <c r="Z119" t="inlineStr"/>
+      <c r="AA119" t="inlineStr"/>
+      <c r="AB119" t="inlineStr"/>
+      <c r="AC119" t="inlineStr"/>
+      <c r="AD119" t="inlineStr"/>
+      <c r="AE119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -11986,6 +12775,12 @@
         </is>
       </c>
       <c r="Y120" t="inlineStr"/>
+      <c r="Z120" t="inlineStr"/>
+      <c r="AA120" t="inlineStr"/>
+      <c r="AB120" t="inlineStr"/>
+      <c r="AC120" t="inlineStr"/>
+      <c r="AD120" t="inlineStr"/>
+      <c r="AE120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -12083,6 +12878,12 @@
         </is>
       </c>
       <c r="Y121" t="inlineStr"/>
+      <c r="Z121" t="inlineStr"/>
+      <c r="AA121" t="inlineStr"/>
+      <c r="AB121" t="inlineStr"/>
+      <c r="AC121" t="inlineStr"/>
+      <c r="AD121" t="inlineStr"/>
+      <c r="AE121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -12180,6 +12981,12 @@
         </is>
       </c>
       <c r="Y122" t="inlineStr"/>
+      <c r="Z122" t="inlineStr"/>
+      <c r="AA122" t="inlineStr"/>
+      <c r="AB122" t="inlineStr"/>
+      <c r="AC122" t="inlineStr"/>
+      <c r="AD122" t="inlineStr"/>
+      <c r="AE122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -12277,6 +13084,12 @@
         </is>
       </c>
       <c r="Y123" t="inlineStr"/>
+      <c r="Z123" t="inlineStr"/>
+      <c r="AA123" t="inlineStr"/>
+      <c r="AB123" t="inlineStr"/>
+      <c r="AC123" t="inlineStr"/>
+      <c r="AD123" t="inlineStr"/>
+      <c r="AE123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -12370,6 +13183,12 @@
       </c>
       <c r="X124" t="inlineStr"/>
       <c r="Y124" t="inlineStr"/>
+      <c r="Z124" t="inlineStr"/>
+      <c r="AA124" t="inlineStr"/>
+      <c r="AB124" t="inlineStr"/>
+      <c r="AC124" t="inlineStr"/>
+      <c r="AD124" t="inlineStr"/>
+      <c r="AE124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -12467,6 +13286,12 @@
         </is>
       </c>
       <c r="Y125" t="inlineStr"/>
+      <c r="Z125" t="inlineStr"/>
+      <c r="AA125" t="inlineStr"/>
+      <c r="AB125" t="inlineStr"/>
+      <c r="AC125" t="inlineStr"/>
+      <c r="AD125" t="inlineStr"/>
+      <c r="AE125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -12564,6 +13389,12 @@
         </is>
       </c>
       <c r="Y126" t="inlineStr"/>
+      <c r="Z126" t="inlineStr"/>
+      <c r="AA126" t="inlineStr"/>
+      <c r="AB126" t="inlineStr"/>
+      <c r="AC126" t="inlineStr"/>
+      <c r="AD126" t="inlineStr"/>
+      <c r="AE126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -12661,6 +13492,12 @@
         </is>
       </c>
       <c r="Y127" t="inlineStr"/>
+      <c r="Z127" t="inlineStr"/>
+      <c r="AA127" t="inlineStr"/>
+      <c r="AB127" t="inlineStr"/>
+      <c r="AC127" t="inlineStr"/>
+      <c r="AD127" t="inlineStr"/>
+      <c r="AE127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -12758,6 +13595,12 @@
         </is>
       </c>
       <c r="Y128" t="inlineStr"/>
+      <c r="Z128" t="inlineStr"/>
+      <c r="AA128" t="inlineStr"/>
+      <c r="AB128" t="inlineStr"/>
+      <c r="AC128" t="inlineStr"/>
+      <c r="AD128" t="inlineStr"/>
+      <c r="AE128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -12855,6 +13698,12 @@
         </is>
       </c>
       <c r="Y129" t="inlineStr"/>
+      <c r="Z129" t="inlineStr"/>
+      <c r="AA129" t="inlineStr"/>
+      <c r="AB129" t="inlineStr"/>
+      <c r="AC129" t="inlineStr"/>
+      <c r="AD129" t="inlineStr"/>
+      <c r="AE129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -12952,6 +13801,12 @@
         </is>
       </c>
       <c r="Y130" t="inlineStr"/>
+      <c r="Z130" t="inlineStr"/>
+      <c r="AA130" t="inlineStr"/>
+      <c r="AB130" t="inlineStr"/>
+      <c r="AC130" t="inlineStr"/>
+      <c r="AD130" t="inlineStr"/>
+      <c r="AE130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -13049,6 +13904,20 @@
         </is>
       </c>
       <c r="Y131" t="inlineStr"/>
+      <c r="Z131" t="inlineStr"/>
+      <c r="AA131" t="inlineStr">
+        <is>
+          <t>genAI = true</t>
+        </is>
+      </c>
+      <c r="AB131" t="inlineStr">
+        <is>
+          <t>AI governance applies to generative AI workloads</t>
+        </is>
+      </c>
+      <c r="AC131" t="inlineStr"/>
+      <c r="AD131" t="inlineStr"/>
+      <c r="AE131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -13146,6 +14015,12 @@
         </is>
       </c>
       <c r="Y132" t="inlineStr"/>
+      <c r="Z132" t="inlineStr"/>
+      <c r="AA132" t="inlineStr"/>
+      <c r="AB132" t="inlineStr"/>
+      <c r="AC132" t="inlineStr"/>
+      <c r="AD132" t="inlineStr"/>
+      <c r="AE132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -13243,6 +14118,12 @@
         </is>
       </c>
       <c r="Y133" t="inlineStr"/>
+      <c r="Z133" t="inlineStr"/>
+      <c r="AA133" t="inlineStr"/>
+      <c r="AB133" t="inlineStr"/>
+      <c r="AC133" t="inlineStr"/>
+      <c r="AD133" t="inlineStr"/>
+      <c r="AE133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -13340,6 +14221,12 @@
         </is>
       </c>
       <c r="Y134" t="inlineStr"/>
+      <c r="Z134" t="inlineStr"/>
+      <c r="AA134" t="inlineStr"/>
+      <c r="AB134" t="inlineStr"/>
+      <c r="AC134" t="inlineStr"/>
+      <c r="AD134" t="inlineStr"/>
+      <c r="AE134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -13437,6 +14324,12 @@
         </is>
       </c>
       <c r="Y135" t="inlineStr"/>
+      <c r="Z135" t="inlineStr"/>
+      <c r="AA135" t="inlineStr"/>
+      <c r="AB135" t="inlineStr"/>
+      <c r="AC135" t="inlineStr"/>
+      <c r="AD135" t="inlineStr"/>
+      <c r="AE135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -13534,6 +14427,12 @@
         </is>
       </c>
       <c r="Y136" t="inlineStr"/>
+      <c r="Z136" t="inlineStr"/>
+      <c r="AA136" t="inlineStr"/>
+      <c r="AB136" t="inlineStr"/>
+      <c r="AC136" t="inlineStr"/>
+      <c r="AD136" t="inlineStr"/>
+      <c r="AE136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -13631,6 +14530,12 @@
         </is>
       </c>
       <c r="Y137" t="inlineStr"/>
+      <c r="Z137" t="inlineStr"/>
+      <c r="AA137" t="inlineStr"/>
+      <c r="AB137" t="inlineStr"/>
+      <c r="AC137" t="inlineStr"/>
+      <c r="AD137" t="inlineStr"/>
+      <c r="AE137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -13728,6 +14633,12 @@
         </is>
       </c>
       <c r="Y138" t="inlineStr"/>
+      <c r="Z138" t="inlineStr"/>
+      <c r="AA138" t="inlineStr"/>
+      <c r="AB138" t="inlineStr"/>
+      <c r="AC138" t="inlineStr"/>
+      <c r="AD138" t="inlineStr"/>
+      <c r="AE138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -13825,6 +14736,12 @@
         </is>
       </c>
       <c r="Y139" t="inlineStr"/>
+      <c r="Z139" t="inlineStr"/>
+      <c r="AA139" t="inlineStr"/>
+      <c r="AB139" t="inlineStr"/>
+      <c r="AC139" t="inlineStr"/>
+      <c r="AD139" t="inlineStr"/>
+      <c r="AE139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -13922,6 +14839,12 @@
         </is>
       </c>
       <c r="Y140" t="inlineStr"/>
+      <c r="Z140" t="inlineStr"/>
+      <c r="AA140" t="inlineStr"/>
+      <c r="AB140" t="inlineStr"/>
+      <c r="AC140" t="inlineStr"/>
+      <c r="AD140" t="inlineStr"/>
+      <c r="AE140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -14019,6 +14942,12 @@
         </is>
       </c>
       <c r="Y141" t="inlineStr"/>
+      <c r="Z141" t="inlineStr"/>
+      <c r="AA141" t="inlineStr"/>
+      <c r="AB141" t="inlineStr"/>
+      <c r="AC141" t="inlineStr"/>
+      <c r="AD141" t="inlineStr"/>
+      <c r="AE141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -14116,6 +15045,12 @@
         </is>
       </c>
       <c r="Y142" t="inlineStr"/>
+      <c r="Z142" t="inlineStr"/>
+      <c r="AA142" t="inlineStr"/>
+      <c r="AB142" t="inlineStr"/>
+      <c r="AC142" t="inlineStr"/>
+      <c r="AD142" t="inlineStr"/>
+      <c r="AE142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -14209,6 +15144,12 @@
       </c>
       <c r="X143" t="inlineStr"/>
       <c r="Y143" t="inlineStr"/>
+      <c r="Z143" t="inlineStr"/>
+      <c r="AA143" t="inlineStr"/>
+      <c r="AB143" t="inlineStr"/>
+      <c r="AC143" t="inlineStr"/>
+      <c r="AD143" t="inlineStr"/>
+      <c r="AE143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -14306,6 +15247,12 @@
         </is>
       </c>
       <c r="Y144" t="inlineStr"/>
+      <c r="Z144" t="inlineStr"/>
+      <c r="AA144" t="inlineStr"/>
+      <c r="AB144" t="inlineStr"/>
+      <c r="AC144" t="inlineStr"/>
+      <c r="AD144" t="inlineStr"/>
+      <c r="AE144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -14403,6 +15350,12 @@
         </is>
       </c>
       <c r="Y145" t="inlineStr"/>
+      <c r="Z145" t="inlineStr"/>
+      <c r="AA145" t="inlineStr"/>
+      <c r="AB145" t="inlineStr"/>
+      <c r="AC145" t="inlineStr"/>
+      <c r="AD145" t="inlineStr"/>
+      <c r="AE145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -14500,6 +15453,12 @@
         </is>
       </c>
       <c r="Y146" t="inlineStr"/>
+      <c r="Z146" t="inlineStr"/>
+      <c r="AA146" t="inlineStr"/>
+      <c r="AB146" t="inlineStr"/>
+      <c r="AC146" t="inlineStr"/>
+      <c r="AD146" t="inlineStr"/>
+      <c r="AE146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -14597,6 +15556,12 @@
         </is>
       </c>
       <c r="Y147" t="inlineStr"/>
+      <c r="Z147" t="inlineStr"/>
+      <c r="AA147" t="inlineStr"/>
+      <c r="AB147" t="inlineStr"/>
+      <c r="AC147" t="inlineStr"/>
+      <c r="AD147" t="inlineStr"/>
+      <c r="AE147" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19803,7 +20768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -19814,6 +20779,10 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19857,6 +20826,26 @@
           <t>Help</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Shown When</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Derivation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -19895,6 +20884,16 @@
           <t>Sets the baseline task list. Exactly one.</t>
         </is>
       </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -19929,6 +20928,16 @@
           <t>Kickoff, requirements gathering, peer review, stakeholder validation, ARB.</t>
         </is>
       </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -19963,6 +20972,16 @@
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>discovery = true</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -19997,6 +21016,16 @@
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>discovery = true</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -20031,6 +21060,16 @@
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>discovery = true</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -20065,6 +21104,16 @@
           <t>Triggers TPRM and vendor onboarding.</t>
         </is>
       </c>
+      <c r="I7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -20095,6 +21144,16 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -20125,6 +21184,16 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -20159,6 +21228,16 @@
           <t>Adds the AI governance chain.</t>
         </is>
       </c>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -20193,6 +21272,16 @@
           <t>Pre-approved modules, so several reviews stop applying.</t>
         </is>
       </c>
+      <c r="I11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -20223,6 +21312,16 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>3</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -20253,6 +21352,16 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -20287,6 +21396,16 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -20321,6 +21440,16 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -20351,6 +21480,16 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -20381,6 +21520,24 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>tier IN ["Tier 0", "Tier 1", "Tier 2", "Tier 3"]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20388,6 +21545,114 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rule ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Expression</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Means</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Why It Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>R_Sourcing</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>newVendor = true OR hardware = true OR newLicense = true</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>any commercial sourcing is involved</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TPRM, contracting and purchasing all hang off this one fact</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>R_SelectionNeeded</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>rfi = true OR rfp = true OR poc = true</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>a product selection route is in play</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>keeps the discovery gates on one switch instead of three</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R_TopTier</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>tier IN ["Tier 0", "Tier 1"]</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>the top service tiers</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>drives the deeper resilience and security scrutiny</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20945,7 +22210,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27771,7 +29036,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27898,7 +29163,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>